<commit_message>
Fixes bug with SFBS data load, test assessment run
</commit_message>
<xml_diff>
--- a/data_raw/smelt/SFBS_2025.xlsx
+++ b/data_raw/smelt/SFBS_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/RTO/WY26/Weekly_assessments/26.02.23/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lmccormick_usbr_gov/Documents/Documents/Research/R/samt_smt_assessments/data_raw/smelt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FDA146F-F8C2-4E00-8FE0-F292F5D2379B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{9FDA146F-F8C2-4E00-8FE0-F292F5D2379B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12894297-B962-469E-8CE8-A789874D0BA4}"/>
   <bookViews>
-    <workbookView xWindow="-15480" yWindow="-13920" windowWidth="23040" windowHeight="12120" xr2:uid="{E6B263F6-6BD8-4845-A7D3-38BD6C57D086}"/>
+    <workbookView xWindow="-11076" yWindow="-14616" windowWidth="21192" windowHeight="11460" xr2:uid="{E6B263F6-6BD8-4845-A7D3-38BD6C57D086}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -845,6 +845,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3EAB52-37DA-4907-ABCB-CFF3844AE140}">
   <dimension ref="A1:M1520"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="19.44140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>